<commit_message>
adding all week 5 modules to git
</commit_message>
<xml_diff>
--- a/Handson/DN - Java FSE Mandatory hands-on detail (1).xlsx
+++ b/Handson/DN - Java FSE Mandatory hands-on detail (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\WEEK\Digital-Nature\Handson\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8AB9F0C-F670-4F01-AE44-365FC6865511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D3F725-5A36-404D-BE72-35CCC6424307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{E078EC40-2268-4F4F-B14B-9403122955B8}"/>
   </bookViews>
@@ -482,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -490,12 +490,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -542,6 +536,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -887,20 +889,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="22"/>
-      <c r="D1" s="23" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="E1" s="24"/>
+      <c r="E1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="16"/>
+      <c r="A2" s="14"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -921,12 +923,12 @@
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>93</v>
       </c>
     </row>
@@ -937,7 +939,7 @@
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="4"/>
@@ -950,12 +952,12 @@
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="8" t="s">
         <v>94</v>
       </c>
     </row>
@@ -966,7 +968,7 @@
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="4"/>
@@ -979,7 +981,7 @@
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="4"/>
@@ -992,7 +994,7 @@
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="4"/>
@@ -1005,7 +1007,7 @@
       <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="7" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="4"/>
@@ -1018,33 +1020,33 @@
       <c r="B10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="7" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="18"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="12" t="s">
+      <c r="A12" s="16"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
     </row>
     <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
@@ -1085,242 +1087,242 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:6" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13" t="s">
+      <c r="D16" s="11"/>
+      <c r="E16" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+    <row r="17" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13" t="s">
+      <c r="D17" s="11"/>
+      <c r="E17" s="11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13" t="s">
+      <c r="D18" s="11"/>
+      <c r="E18" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+    <row r="20" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="13" t="s">
+    <row r="21" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="13" t="s">
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="14" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:5" s="12" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="13" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="13" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="13" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-    </row>
-    <row r="27" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="13" t="s">
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+    </row>
+    <row r="27" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-    </row>
-    <row r="28" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+    </row>
+    <row r="28" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-    </row>
-    <row r="29" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+    </row>
+    <row r="29" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-    </row>
-    <row r="30" spans="1:5" s="14" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="13" t="s">
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+    </row>
+    <row r="30" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-    </row>
-    <row r="31" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+    </row>
+    <row r="31" spans="1:5" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="C31" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="17" t="s">
+      <c r="D31" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E31" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="18"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="6" t="s">
+    <row r="32" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="24"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="10" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1552,17 +1554,17 @@
       <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="7" t="s">
+      <c r="A48" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C48" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
+      <c r="C48" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1583,15 +1585,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6f516c4-2602-422c-aa9a-755893ba4f98">
@@ -1600,6 +1593,15 @@
     <TaxCatchAll xmlns="3c35e321-f73a-4dae-ae38-a0459de24735"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1863,14 +1865,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F0F638-0648-46BA-B1DF-3E4F6ADB00E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B84191-BBE7-412A-A5F6-7B8D27AECA6C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -1884,6 +1878,14 @@
     <ds:schemaRef ds:uri="951c5514-b77c-4532-82d5-a05f2f7d58e2"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F0F638-0648-46BA-B1DF-3E4F6ADB00E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>